<commit_message>
Added landing Page and preloader
</commit_message>
<xml_diff>
--- a/dashboard/backend/src/data/candidates.xlsx
+++ b/dashboard/backend/src/data/candidates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahes\Desktop\technologia_round2\round_2\dashboard\backend\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E344586F-C63B-47E5-BFFC-C631087C2907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D6E0BB-8312-4CA9-BC10-94135FBB6A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
     <t>score</t>
   </si>
   <si>
-    <t>Aarav Sharma</t>
-  </si>
-  <si>
     <t>aarav.sharma@example.com</t>
   </si>
   <si>
@@ -92,6 +89,9 @@
   </si>
   <si>
     <t>tn105</t>
+  </si>
+  <si>
+    <t>Aarav Mishra</t>
   </si>
 </sst>
 </file>
@@ -375,16 +375,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>7</v>
       </c>
       <c r="E2" s="1">
         <v>88</v>
@@ -392,16 +392,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="E3" s="1">
         <v>92</v>
@@ -409,16 +409,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="E4" s="1">
         <v>76</v>
@@ -426,16 +426,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E5" s="1">
         <v>95</v>
@@ -443,16 +443,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="E6" s="1">
         <v>81</v>

</xml_diff>